<commit_message>
client: nhãn Thuyền/Guild khỏi đè, thẻ màu nhiều từ, mô tả thử thách sinh từ cột luật, rà tên tướng
</commit_message>
<xml_diff>
--- a/server/excel/release/blessed-grotto.xlsx
+++ b/server/excel/release/blessed-grotto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="我的洞天福地" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="掠夺" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="稀有道具掠夺概率" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="我的洞天福地" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掠夺" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="稀有道具掠夺概率" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="299">
   <si>
     <t xml:space="preserve">等级</t>
   </si>
@@ -179,589 +179,601 @@
     <t xml:space="preserve">Kiếm Trủng cấp thấp khoáng mạch</t>
   </si>
   <si>
+    <t xml:space="preserve">Khoáng mạch cấp thấp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1002:30#1005:30#1006:30#1007:30#1008:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:18 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hs_bg4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:908#0:4:908</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battle_bg2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:19 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:957#0:4:957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:20 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:1007#0:4:1007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiếm Trủng trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khoáng mạch trung cấp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:21 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1056#0:4:1056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:22 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1106#0:4:1106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:23 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1155#0:4:1155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiếm Trủng cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khoáng mạch cao cấp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:24 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1205#0:4:1205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:25 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1254#0:4:1254</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:26 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1304#0:4:1304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiếm Trủng long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:27 #1014:5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:12#0:0:1353#0:4:1353</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Đình Mật Đạo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Đình cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:974#0:4:974</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battle_bg1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:21 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1023#0:4:1023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:22 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1073#0:4:1073</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Đình trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1122#0:4:1122</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:24 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1172#0:4:1172</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:25 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1221#0:4:1221</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Đình cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:26 #1014:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1271#0:4:1271</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:27 #1014:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1320#0:4:1320</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:28 #1014:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1370#0:4:1370</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Đình long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:29 #1014:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:14#0:0:1419#0:4:1419</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vạn Pháp Yêu Thành</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yêu thành cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1040#0:4:1040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battle_bg3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1089#0:4:1089</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:23 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1139#0:4:1139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yêu thành trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1188#0:4:1188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1238#0:4:1238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:26 #1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1287#0:4:1287</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yêu thành cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:27 #1014:2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1337#0:4:1337</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:28 #1014:2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1386#0:4:1386</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:29 #1014:2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1436#0:4:1436</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yêu thành long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:30 #1014:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:16#0:0:1485#0:4:1485</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bồng Lai Tiên Cảnh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bồng Lai cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1106#0:4:1106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battle_bg4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1155#0:4:1155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:9#0:0:1205#0:4:1205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bồng Lai trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:25 #1014:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1254#0:4:1254</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1304#0:4:1304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1353#0:4:1353</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bồng Lai cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:28 #1014:3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:11#0:0:1403#0:4:1403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:29 #1014:3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:11#0:0:1452#0:4:1452</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:30 #1014:3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:11#0:0:1502#0:4:1502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bồng Lai long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:31 #1014:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:18#0:0:1551#0:4:1551</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hồng Quân Di Tích</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hồng Quân cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:24 #1014:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1172#0:4:1172</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battle_bg13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1221#0:4:1221</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1271#0:4:1271</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hồng Quân trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:11#0:0:1320#0:4:1320</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:11#0:0:1370#0:4:1370</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:11#0:0:1419#0:4:1419</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hồng Quân cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:30 #1014:4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:12#0:0:1469#0:4:1469</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:31 #1014:4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:12#0:0:1518#0:4:1518</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:32 #1014:4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:12#0:0:1568#0:4:1568</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hồng Quân long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:33 #1014:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:20#0:0:1617#0:4:1617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trúc Hải Phúc Địa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biển trúc cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:5#0:0:808#0:4:808</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:5#0:0:857#0:4:857</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:5#0:0:900#0:4:900</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biển trúc trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:950#0:4:950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:1000#0:4:1000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:1050#0:4:1050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biển trúc cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1100#0:4:1100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1150#0:4:1150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1200#0:4:1200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biển trúc long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:10#0:0:1250#0:4:1250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thủy Liêm Động Thiên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Màn nước cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:870#0:4:870</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:920#0:4:920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:6#0:0:970#0:4:970</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Màn nước trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1020#0:4:1020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1070#0:4:1070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:7#0:0:1120#0:4:1120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Màn nước cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1170#0:4:1170</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1220#0:4:1220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3:100215:8#0:0:1270#0:4:1270</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Màn nước long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nguyên Thủy Địa Nguyên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nguyên cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nguyên trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nguyên cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nguyên long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nguyên Thủy Thiên Nguyên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Nguyên cấp thấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zi10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bg10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Nguyên trung cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Nguyên cao cấp khoáng mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiên Nguyên long mạch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">物品大类ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">物品ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">被掠夺概率</t>
+  </si>
+  <si>
+    <t xml:space="preserve">荒古剑冢</t>
+  </si>
+  <si>
     <t xml:space="preserve">低级矿脉</t>
   </si>
   <si>
-    <t xml:space="preserve">1002:30#1005:30#1006:30#1007:30#1008:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:18 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hs_bg4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:908#0:4:908</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battle_bg2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:19 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:957#0:4:957</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:20 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:1007#0:4:1007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kiếm Trủng trung cấp khoáng mạch</t>
+    <t xml:space="preserve">荒古</t>
+  </si>
+  <si>
+    <t xml:space="preserve">荒古低级矿脉</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:18 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1014:0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:19 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1011:20 </t>
   </si>
   <si>
     <t xml:space="preserve">中级矿脉</t>
   </si>
   <si>
-    <t xml:space="preserve">1012:21 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1056#0:4:1056</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:22 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1106#0:4:1106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:23 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1155#0:4:1155</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kiếm Trủng cao cấp khoáng mạch</t>
+    <t xml:space="preserve">荒古中级矿脉</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:21 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:22 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012:23 </t>
   </si>
   <si>
     <t xml:space="preserve">高级矿脉</t>
   </si>
   <si>
-    <t xml:space="preserve">1013:24 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1205#0:4:1205</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:25 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1254#0:4:1254</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:26 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1304#0:4:1304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kiếm Trủng long mạch</t>
+    <t xml:space="preserve">荒古高级矿脉</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:24 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:25 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1013:26 </t>
   </si>
   <si>
     <t xml:space="preserve">龙脉</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:27 #1014:5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:12#0:0:1353#0:4:1353</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Đình Mật Đạo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Đình cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:974#0:4:974</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battle_bg1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:21 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1023#0:4:1023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:22 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1073#0:4:1073</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Đình trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1122#0:4:1122</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:24 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1172#0:4:1172</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:25 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1221#0:4:1221</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Đình cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:26 #1014:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1271#0:4:1271</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:27 #1014:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1320#0:4:1320</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:28 #1014:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1370#0:4:1370</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Đình long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:29 #1014:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:14#0:0:1419#0:4:1419</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vạn Pháp Yêu Thành</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yêu thành cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1040#0:4:1040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battle_bg3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1089#0:4:1089</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:23 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1139#0:4:1139</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yêu thành trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1188#0:4:1188</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1238#0:4:1238</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:26 #1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1287#0:4:1287</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yêu thành cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:27 #1014:2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1337#0:4:1337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:28 #1014:2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1386#0:4:1386</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:29 #1014:2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1436#0:4:1436</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yêu thành long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:30 #1014:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:16#0:0:1485#0:4:1485</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bồng Lai Tiên Cảnh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bồng Lai cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1106#0:4:1106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battle_bg4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1155#0:4:1155</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:9#0:0:1205#0:4:1205</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bồng Lai trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:25 #1014:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1254#0:4:1254</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1304#0:4:1304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1353#0:4:1353</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bồng Lai cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:28 #1014:3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:11#0:0:1403#0:4:1403</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:29 #1014:3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:11#0:0:1452#0:4:1452</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:30 #1014:3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:11#0:0:1502#0:4:1502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bồng Lai long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:31 #1014:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:18#0:0:1551#0:4:1551</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hồng Quân Di Tích</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hồng Quân cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:24 #1014:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1172#0:4:1172</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battle_bg13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1221#0:4:1221</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1271#0:4:1271</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hồng Quân trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:11#0:0:1320#0:4:1320</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:11#0:0:1370#0:4:1370</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:11#0:0:1419#0:4:1419</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hồng Quân cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:30 #1014:4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:12#0:0:1469#0:4:1469</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:31 #1014:4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:12#0:0:1518#0:4:1518</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:32 #1014:4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:12#0:0:1568#0:4:1568</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hồng Quân long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:33 #1014:25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:20#0:0:1617#0:4:1617</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trúc Hải Phúc Địa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biển trúc cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:5#0:0:808#0:4:808</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:5#0:0:857#0:4:857</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:5#0:0:900#0:4:900</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biển trúc trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:950#0:4:950</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:1000#0:4:1000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:1050#0:4:1050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biển trúc cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1100#0:4:1100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1150#0:4:1150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1200#0:4:1200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biển trúc long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:10#0:0:1250#0:4:1250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thủy Liêm Động Thiên</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Màn nước cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:870#0:4:870</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:920#0:4:920</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:6#0:0:970#0:4:970</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Màn nước trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1020#0:4:1020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1070#0:4:1070</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:7#0:0:1120#0:4:1120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Màn nước cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1170#0:4:1170</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1220#0:4:1220</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3:100215:8#0:0:1270#0:4:1270</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Màn nước long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nguyên Thủy Địa Nguyên</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nguyên cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nguyên trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nguyên cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nguyên long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nguyên Thủy Thiên Nguyên</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Nguyên cấp thấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zi10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bg10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Nguyên trung cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Nguyên cao cấp khoáng mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thiên Nguyên long mạch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">物品大类ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">物品ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">被掠夺概率</t>
-  </si>
-  <si>
-    <t xml:space="preserve">荒古剑冢</t>
-  </si>
-  <si>
-    <t xml:space="preserve">荒古</t>
-  </si>
-  <si>
-    <t xml:space="preserve">荒古低级矿脉</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:18 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1014:0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:19 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1011:20 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">荒古中级矿脉</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:21 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:22 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012:23 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">荒古高级矿脉</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:24 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:25 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1013:26 </t>
   </si>
   <si>
     <t xml:space="preserve">荒古龙脉</t>
@@ -9032,1151 +9044,1151 @@
         <v>232</v>
       </c>
       <c r="H1" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G2" t="s">
         <v>232</v>
       </c>
       <c r="H2" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C3" t="s">
         <v>238</v>
-      </c>
-      <c r="B3" t="s">
-        <v>236</v>
-      </c>
-      <c r="C3" t="s">
-        <v>237</v>
       </c>
       <c r="G3" t="s">
         <v>232</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G4" t="s">
         <v>232</v>
       </c>
       <c r="H4" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G5" t="s">
         <v>232</v>
       </c>
       <c r="H5" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G6" t="s">
         <v>232</v>
       </c>
       <c r="H6" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G7" t="s">
         <v>232</v>
       </c>
       <c r="H7" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J7" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G8" t="s">
         <v>232</v>
       </c>
       <c r="H8" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J8" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C9" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G9" t="s">
         <v>232</v>
       </c>
       <c r="H9" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I9" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G10" t="s">
         <v>232</v>
       </c>
       <c r="H10" t="s">
-        <v>82</v>
+        <v>251</v>
       </c>
       <c r="I10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J10" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C11" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="G11" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H11" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I11" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J11" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C12" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G12" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H12" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I12" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J12" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C13" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G13" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H13" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I13" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J13" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>259</v>
+      </c>
+      <c r="B14" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" t="s">
+        <v>238</v>
+      </c>
+      <c r="G14" t="s">
         <v>255</v>
       </c>
-      <c r="B14" t="s">
-        <v>236</v>
-      </c>
-      <c r="C14" t="s">
-        <v>237</v>
-      </c>
-      <c r="G14" t="s">
-        <v>251</v>
-      </c>
       <c r="H14" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J14" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G15" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H15" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I15" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J15" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B16" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C16" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G16" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H16" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I16" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J16" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C17" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G17" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H17" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I17" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J17" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C18" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G18" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H18" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I18" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J18" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B19" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C19" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G19" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H19" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I19" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J19" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B20" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C20" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G20" t="s">
+        <v>255</v>
+      </c>
+      <c r="H20" t="s">
         <v>251</v>
       </c>
-      <c r="H20" t="s">
-        <v>82</v>
-      </c>
       <c r="I20" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J20" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C21" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="G21" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H21" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I21" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J21" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B22" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C22" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G22" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H22" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I22" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J22" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="B23" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C23" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G23" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H23" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I23" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J23" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B24" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C24" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G24" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H24" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I24" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J24" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B25" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C25" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G25" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H25" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I25" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J25" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B26" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C26" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G26" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H26" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I26" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J26" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
+        <v>274</v>
+      </c>
+      <c r="B27" t="s">
+        <v>237</v>
+      </c>
+      <c r="C27" t="s">
+        <v>238</v>
+      </c>
+      <c r="G27" t="s">
+        <v>269</v>
+      </c>
+      <c r="H27" t="s">
+        <v>246</v>
+      </c>
+      <c r="I27" t="s">
         <v>270</v>
       </c>
-      <c r="B27" t="s">
-        <v>236</v>
-      </c>
-      <c r="C27" t="s">
-        <v>237</v>
-      </c>
-      <c r="G27" t="s">
-        <v>265</v>
-      </c>
-      <c r="H27" t="s">
-        <v>74</v>
-      </c>
-      <c r="I27" t="s">
-        <v>266</v>
-      </c>
       <c r="J27" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B28" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C28" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="G28" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H28" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I28" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J28" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B29" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C29" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="G29" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H29" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I29" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J29" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B30" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C30" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="G30" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H30" t="s">
-        <v>82</v>
+        <v>251</v>
       </c>
       <c r="I30" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="J30" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B31" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C31" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="G31" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H31" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I31" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J31" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C32" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G32" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H32" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I32" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J32" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G33" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H33" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I33" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J33" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B34" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C34" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G34" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H34" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I34" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J34" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B35" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C35" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G35" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H35" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I35" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J35" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B36" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C36" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G36" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H36" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I36" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J36" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B37" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C37" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G37" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H37" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I37" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="J37" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B38" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C38" t="s">
+        <v>285</v>
+      </c>
+      <c r="G38" t="s">
+        <v>280</v>
+      </c>
+      <c r="H38" t="s">
+        <v>246</v>
+      </c>
+      <c r="I38" t="s">
         <v>281</v>
       </c>
-      <c r="G38" t="s">
-        <v>276</v>
-      </c>
-      <c r="H38" t="s">
-        <v>74</v>
-      </c>
-      <c r="I38" t="s">
-        <v>277</v>
-      </c>
       <c r="J38" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B39" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C39" t="s">
+        <v>285</v>
+      </c>
+      <c r="G39" t="s">
+        <v>280</v>
+      </c>
+      <c r="H39" t="s">
+        <v>246</v>
+      </c>
+      <c r="I39" t="s">
         <v>281</v>
       </c>
-      <c r="G39" t="s">
-        <v>276</v>
-      </c>
-      <c r="H39" t="s">
-        <v>74</v>
-      </c>
-      <c r="I39" t="s">
-        <v>277</v>
-      </c>
       <c r="J39" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B40" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C40" t="s">
+        <v>285</v>
+      </c>
+      <c r="G40" t="s">
+        <v>280</v>
+      </c>
+      <c r="H40" t="s">
+        <v>251</v>
+      </c>
+      <c r="I40" t="s">
         <v>281</v>
       </c>
-      <c r="G40" t="s">
-        <v>276</v>
-      </c>
-      <c r="H40" t="s">
-        <v>82</v>
-      </c>
-      <c r="I40" t="s">
-        <v>277</v>
-      </c>
       <c r="J40" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B41" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C41" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="G41" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="H41" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I41" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J41" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B42" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C42" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G42" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="H42" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I42" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J42" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B43" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C43" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G43" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="H43" t="s">
-        <v>53</v>
+        <v>233</v>
       </c>
       <c r="I43" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J43" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B44" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C44" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="G44" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="H44" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I44" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J44" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B45" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C45" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="G45" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="H45" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I45" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J45" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B46" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C46" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="G46" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="H46" t="s">
-        <v>66</v>
+        <v>241</v>
       </c>
       <c r="I46" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J46" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B47" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C47" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="G47" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="H47" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="I47" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J47" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B48" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C48" t="s">
+        <v>294</v>
+      </c>
+      <c r="G48" t="s">
+        <v>289</v>
+      </c>
+      <c r="H48" t="s">
+        <v>246</v>
+      </c>
+      <c r="I48" t="s">
         <v>290</v>
       </c>
-      <c r="G48" t="s">
-        <v>285</v>
-      </c>
-      <c r="H48" t="s">
-        <v>74</v>
-      </c>
-      <c r="I48" t="s">
-        <v>286</v>
-      </c>
       <c r="J48" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B49" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C49" t="s">
+        <v>294</v>
+      </c>
+      <c r="G49" t="s">
+        <v>289</v>
+      </c>
+      <c r="H49" t="s">
+        <v>246</v>
+      </c>
+      <c r="I49" t="s">
         <v>290</v>
       </c>
-      <c r="G49" t="s">
-        <v>285</v>
-      </c>
-      <c r="H49" t="s">
-        <v>74</v>
-      </c>
-      <c r="I49" t="s">
-        <v>286</v>
-      </c>
       <c r="J49" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B50" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C50" t="s">
+        <v>294</v>
+      </c>
+      <c r="G50" t="s">
+        <v>289</v>
+      </c>
+      <c r="H50" t="s">
+        <v>251</v>
+      </c>
+      <c r="I50" t="s">
         <v>290</v>
       </c>
-      <c r="G50" t="s">
-        <v>285</v>
-      </c>
-      <c r="H50" t="s">
-        <v>82</v>
-      </c>
-      <c r="I50" t="s">
-        <v>286</v>
-      </c>
       <c r="J50" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B51" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C51" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>